<commit_message>
Add academic year closure page and pagination views
- Created a new Blade view for closing the academic year with a form to select the target year/semester and confirm the action.
- Implemented dynamic warning messages based on the selected target.
- Added pagination views for Bootstrap 4, Bootstrap 5, Semantic UI, and Tailwind CSS to enhance pagination functionality across the application.
- Included simple pagination views for Bootstrap and Tailwind CSS for streamlined navigation.
</commit_message>
<xml_diff>
--- a/public/templates/import-ekstrakurikuler.xlsx
+++ b/public/templates/import-ekstrakurikuler.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AdM\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\ekskulio\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{730F26CC-5685-4578-BB62-258873E2E1EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7122A00-7649-4A9F-BBF6-19773ED52957}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="768" yWindow="768" windowWidth="21600" windowHeight="11232" xr2:uid="{CDC1ACF0-9087-4BBD-A3C1-E4B7A3B0C523}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CDC1ACF0-9087-4BBD-A3C1-E4B7A3B0C523}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="27">
   <si>
     <t>id</t>
   </si>
@@ -42,12 +42,6 @@
     <t>nama_ekstrakurikuler</t>
   </si>
   <si>
-    <t>kode</t>
-  </si>
-  <si>
-    <t>category_id</t>
-  </si>
-  <si>
     <t>deskripsi</t>
   </si>
   <si>
@@ -57,9 +51,6 @@
     <t>status</t>
   </si>
   <si>
-    <t>user_id</t>
-  </si>
-  <si>
     <t>hari</t>
   </si>
   <si>
@@ -100,101 +91,7 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">2. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">user_id </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">diisi jika ingin langsung mencocokkan dengan id pembina (tabel </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>users</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>).</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">1. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">category_id </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">diisi jika ingin langsung mencocokkan dengan id kategori ekstrakurikuler (tabel </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>extracurricular_categories</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>).</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">3. </t>
+      <t xml:space="preserve">4. </t>
     </r>
     <r>
       <rPr>
@@ -218,12 +115,105 @@
       <t>diisi dengan separator koma tanpa spasi.</t>
     </r>
   </si>
+  <si>
+    <r>
+      <t xml:space="preserve">1. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">kode_ekstrakurikuler </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>bersifat opsional. Jika kosong, maka akan di-generate oleh sistem.</t>
+    </r>
+  </si>
+  <si>
+    <t>kode_ekstrakurikuler</t>
+  </si>
+  <si>
+    <t>kode_kategori_ekstrakurikuler</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">2. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">kode_kategori_ekstrakurikuler </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>diisi jika ingin langsung mencocokkan dengan kategori ekstrakurikuler.</t>
+    </r>
+  </si>
+  <si>
+    <t>email_pembina</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">3. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">email_pembina </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>diisi jika ingin langsung mencocokkan dengan akun pembina.</t>
+    </r>
+  </si>
+  <si>
+    <t>pembina@ekskulio.test</t>
+  </si>
+  <si>
+    <t>ODB</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -239,6 +229,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -248,7 +246,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -256,18 +254,59 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -580,21 +619,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{865C1D33-BA53-4B78-BF39-5FAA9EC9879E}">
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:AF8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.88671875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.21875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.33203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="30.109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12.109375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -602,107 +641,187 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="G1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>20</v>
-      </c>
+      <c r="K1" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="L1" s="6"/>
+      <c r="M1" s="6"/>
+      <c r="N1" s="6"/>
+      <c r="O1" s="6"/>
+      <c r="P1" s="6"/>
+      <c r="Q1" s="6"/>
+      <c r="R1" s="6"/>
+      <c r="S1" s="6"/>
+      <c r="T1" s="6"/>
+      <c r="U1" s="6"/>
+      <c r="V1" s="6"/>
+      <c r="W1" s="6"/>
+      <c r="X1" s="6"/>
+      <c r="Y1" s="6"/>
+      <c r="Z1" s="6"/>
+      <c r="AA1" s="6"/>
+      <c r="AB1" s="6"/>
+      <c r="AC1" s="6"/>
+      <c r="AD1" s="6"/>
+      <c r="AE1" s="6"/>
+      <c r="AF1" s="6"/>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>43</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>18</v>
+        <v>15</v>
+      </c>
+      <c r="D2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="F2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2" t="s">
         <v>9</v>
       </c>
-      <c r="G2" t="s">
-        <v>10</v>
-      </c>
-      <c r="H2" t="s">
-        <v>11</v>
-      </c>
-      <c r="I2" t="s">
-        <v>12</v>
-      </c>
-      <c r="K2" t="s">
-        <v>22</v>
-      </c>
+      <c r="K2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
+      <c r="O2" s="3"/>
+      <c r="P2" s="3"/>
+      <c r="Q2" s="3"/>
+      <c r="R2" s="3"/>
+      <c r="S2" s="3"/>
+      <c r="T2" s="3"/>
+      <c r="U2" s="3"/>
+      <c r="V2" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="W2" s="3"/>
+      <c r="X2" s="3"/>
+      <c r="Y2" s="3"/>
+      <c r="Z2" s="3"/>
+      <c r="AA2" s="3"/>
+      <c r="AB2" s="3"/>
+      <c r="AC2" s="3"/>
+      <c r="AD2" s="3"/>
+      <c r="AE2" s="3"/>
+      <c r="AF2" s="3"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>44</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H3" t="s">
+        <v>8</v>
+      </c>
+      <c r="I3" t="s">
         <v>13</v>
       </c>
-      <c r="C3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H3" t="s">
-        <v>11</v>
-      </c>
-      <c r="I3" t="s">
-        <v>16</v>
-      </c>
-      <c r="K3" t="s">
-        <v>21</v>
-      </c>
+      <c r="K3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+      <c r="N3" s="3"/>
+      <c r="O3" s="3"/>
+      <c r="P3" s="3"/>
+      <c r="Q3" s="3"/>
+      <c r="R3" s="3"/>
+      <c r="S3" s="3"/>
+      <c r="T3" s="3"/>
+      <c r="U3" s="3"/>
+      <c r="V3" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="W3" s="3"/>
+      <c r="X3" s="3"/>
+      <c r="Y3" s="3"/>
+      <c r="Z3" s="3"/>
+      <c r="AA3" s="3"/>
+      <c r="AB3" s="3"/>
+      <c r="AC3" s="3"/>
+      <c r="AD3" s="3"/>
+      <c r="AE3" s="3"/>
+      <c r="AF3" s="3"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
-      <c r="K4" t="s">
-        <v>23</v>
-      </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
     </row>
   </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="K3:U3"/>
+    <mergeCell ref="V2:AF2"/>
+    <mergeCell ref="V3:AF3"/>
+    <mergeCell ref="K2:U2"/>
+    <mergeCell ref="K1:AF1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{A2D90C6A-5B71-4F7E-B56C-9CA4C56B1ECF}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>